<commit_message>
data: update 2026-05-28 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-19</v>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>-15</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.03</v>
+        <v>0</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>-9</v>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.39</v>
+        <v>0</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>5</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.25</v>
+        <v>0</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>0</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="E39" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="E42" s="24" t="n">
-        <v>3.65</v>
+        <v>0</v>
       </c>
       <c r="F42" s="24" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.63</v>
+        <v>0</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>3</v>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3129.56</v>
+        <v>0</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-172.15</v>
+        <v>0</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.51</v>
+        <v>0</v>
       </c>
       <c r="F66" s="24" t="n">
         <v>-36</v>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=13.0bp [OK]
-HY OAS 5dd=14.0bp
+          <t>HY OAS 20dd=Nonebp [OK]
+HY OAS 5dd=Nonebp
 HYG 5d=0.8% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=-0.3% [OK]

</xml_diff>

<commit_message>
data: update 2026-06-19 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -2916,10 +2916,10 @@
         <is>
           <t>HY OAS 20dd=15.0bp [OK]
 HY OAS 5dd=17.0bp
-HYG 5d=0.3% [OK]
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.1% [OK]
-SPY vs 200MA: above ($SPY=740.9600219726562, 200MA=685.7)
+FXY 5d=nan% [OK]
+SPY vs 200MA: above ($SPY=746.739990234375, 200MA=684.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-06-22 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>44</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.23</v>
+        <v>2.21</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-5</v>
+        <v>-8</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.49</v>
+        <v>4.46</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.93</v>
+        <v>4.9</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.23</v>
+        <v>2.18</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>-12</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>-11</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-12</v>
@@ -1984,7 +1984,7 @@
         <v>74</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-24</v>
+        <v>-15</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,11 +2914,11 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=15.0bp [OK]
-HY OAS 5dd=17.0bp
+          <t>HY OAS 20dd=8.0bp [OK]
+HY OAS 5dd=5.0bp
 HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=nan% [OK]
+FXY 5d=-1.0% [OK]
 SPY vs 200MA: above ($SPY=746.739990234375, 200MA=684.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>

</xml_diff>

<commit_message>
data: update 2026-06-23 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>44</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>27</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>71</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.21</v>
+        <v>2.28</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.46</v>
+        <v>4.51</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.9</v>
+        <v>4.95</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.23</v>
+        <v>2.21</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.18</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.61</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>7</v>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=8.0bp [OK]
-HY OAS 5dd=5.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=7.0bp [OK]
+HY OAS 5dd=1.0bp
+HYG 5d=0.0% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-1.0% [OK]
-SPY vs 200MA: above ($SPY=746.739990234375, 200MA=684.5)
+FXY 5d=-0.8% [OK]
+SPY vs 200MA: above ($SPY=744.3900146484375, 200MA=685.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-06-24 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>44</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.28</v>
+        <v>2.29</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-13</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.51</v>
+        <v>4.5</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>6</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.95</v>
+        <v>4.94</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.21</v>
+        <v>2.18</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.61</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=7.0bp [OK]
-HY OAS 5dd=1.0bp
-HYG 5d=0.0% [OK]
+          <t>HY OAS 20dd=0.0bp [OK]
+HY OAS 5dd=0.0bp
+HYG 5d=-0.2% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=-0.8% [OK]
-SPY vs 200MA: above ($SPY=744.3900146484375, 200MA=685.0)
+SPY vs 200MA: above ($SPY=733.5800170898438, 200MA=685.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-06-25 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.29</v>
+        <v>2.23</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-13</v>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.5</v>
+        <v>4.41</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.94</v>
+        <v>4.86</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.18</v>
+        <v>2.21</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-7</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-6</v>
+        <v>2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-7</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3033.44</v>
+        <v>2951.42</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-131.84</v>
+        <v>-26.25</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.47</v>
+        <v>6.49</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-37</v>
+        <v>-38</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=0.0bp [OK]
-HY OAS 5dd=0.0bp
+          <t>HY OAS 20dd=-4.0bp [OK]
+HY OAS 5dd=-13.0bp
 HYG 5d=-0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.8% [OK]
-SPY vs 200MA: above ($SPY=733.5800170898438, 200MA=685.5)
+FXY 5d=-0.9% [OK]
+SPY vs 200MA: above ($SPY=733.239990234375, 200MA=685.9)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-06-26 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.23</v>
+        <v>2.19</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-13</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1096,7 +1096,7 @@
         <v>4.86</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.19</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>-0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-15</v>
+        <v>-19</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-4.0bp [OK]
-HY OAS 5dd=-13.0bp
-HYG 5d=-0.2% [OK]
+          <t>HY OAS 20dd=-6.0bp [OK]
+HY OAS 5dd=-12.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.9% [OK]
-SPY vs 200MA: above ($SPY=733.239990234375, 200MA=685.9)
+FXY 5d=-0.7% [OK]
+SPY vs 200MA: above ($SPY=734.2999877929688, 200MA=686.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-06-29 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.19</v>
+        <v>2.18</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-12</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.4</v>
+        <v>4.38</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.86</v>
+        <v>4.87</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.2</v>
+        <v>2.22</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F40" s="24" t="n">
         <v>1</v>
-      </c>
-      <c r="F40" s="24" t="n">
-        <v>-0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-6</v>
+        <v>-9</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-6.0bp [OK]
-HY OAS 5dd=-12.0bp
-HYG 5d=0.2% [OK]
+          <t>HY OAS 20dd=-9.0bp [OK]
+HY OAS 5dd=-17.0bp
+HYG 5d=-0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.7% [OK]
-SPY vs 200MA: above ($SPY=734.2999877929688, 200MA=686.4)
+FXY 5d=-0.2% [OK]
+SPY vs 200MA: above ($SPY=728.989990234375, 200MA=686.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-06-30 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.18</v>
+        <v>2.16</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.87</v>
+        <v>4.86</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.22</v>
+        <v>2.24</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>16</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.2</v>
+        <v>2.22</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>4</v>
@@ -1624,7 +1624,7 @@
         <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-9.0bp [OK]
-HY OAS 5dd=-17.0bp
-HYG 5d=-0.2% [OK]
+          <t>HY OAS 20dd=-8.0bp [OK]
+HY OAS 5dd=-15.0bp
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=-0.2% [OK]
-SPY vs 200MA: above ($SPY=728.989990234375, 200MA=686.8)
+SPY vs 200MA: above ($SPY=741.0, 200MA=687.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-01 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>72</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.16</v>
+        <v>2.2</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-9</v>
+        <v>-13</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.38</v>
+        <v>4.44</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.86</v>
+        <v>4.91</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>16</v>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.22</v>
+        <v>2.2</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>-3</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.68</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>76</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-8.0bp [OK]
-HY OAS 5dd=-15.0bp
+          <t>HY OAS 20dd=-4.0bp [OK]
+HY OAS 5dd=-4.0bp
 HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.2% [OK]
-SPY vs 200MA: above ($SPY=741.0, 200MA=687.3)
+FXY 5d=-0.6% [OK]
+SPY vs 200MA: above ($SPY=746.77001953125, 200MA=687.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-02 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-13</v>
+        <v>-18</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.44</v>
+        <v>4.48</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>3</v>
+        <v>-2</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.91</v>
+        <v>4.97</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.23</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.2</v>
+        <v>2.22</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>-3</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>-2</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.68</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-3</v>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2951.42</v>
+        <v>2966.9</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-26.25</v>
+        <v>-27.34</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>146</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.49</v>
+        <v>6.43</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-38</v>
+        <v>-34</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-4.0bp [OK]
-HY OAS 5dd=-4.0bp
+          <t>HY OAS 20dd=1.0bp [OK]
+HY OAS 5dd=2.0bp
 HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.6% [OK]
-SPY vs 200MA: above ($SPY=746.77001953125, 200MA=687.8)
+FXY 5d=-0.5% [OK]
+SPY vs 200MA: above ($SPY=745.760009765625, 200MA=688.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-03 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>-3</v>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=1.0bp [OK]
-HY OAS 5dd=2.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=-1.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.5% [OK]
-SPY vs 200MA: above ($SPY=745.760009765625, 200MA=688.3)
+FXY 5d=0.5% [OK]
+SPY vs 200MA: above ($SPY=744.780029296875, 200MA=688.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-06 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>49</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.25</v>
+        <v>2.26</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-18</v>
+        <v>-15</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.48</v>
+        <v>4.49</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.22</v>
+        <v>2.21</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>-3</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>-2</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-19</v>
+        <v>6</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=3.0bp
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=9.0bp
 HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=0.5% [OK]

</xml_diff>

<commit_message>
data: update 2026-07-07 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>35</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>2</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.26</v>
+        <v>2.24</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-15</v>
+        <v>-13</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.49</v>
+        <v>4.48</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.98</v>
+        <v>4.99</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>-1</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.63</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>75</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=9.0bp
-HYG 5d=0.2% [OK]
+          <t>HY OAS 20dd=3.0bp [OK]
+HY OAS 5dd=8.0bp
+HYG 5d=0.5% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.5% [OK]
-SPY vs 200MA: above ($SPY=744.780029296875, 200MA=688.7)
+FXY 5d=-0.2% [OK]
+SPY vs 200MA: above ($SPY=751.280029296875, 200MA=689.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-08 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>78</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -949,7 +949,7 @@
         <v>86</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>6</v>
+        <v>-2</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.24</v>
+        <v>2.3</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-13</v>
+        <v>-11</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.48</v>
+        <v>4.55</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>4.99</v>
+        <v>5.05</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.25</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.22</v>
+        <v>2.19</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=3.0bp [OK]
+          <t>HY OAS 20dd=11.0bp [OK]
 HY OAS 5dd=8.0bp
-HYG 5d=0.5% [OK]
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.2% [OK]
-SPY vs 200MA: above ($SPY=751.280029296875, 200MA=689.2)
+FXY 5d=-0.1% [OK]
+SPY vs 200MA: above ($SPY=747.7100219726562, 200MA=689.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-09 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Bull Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.55</v>
+        <v>4.56</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>0</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.05</v>
+        <v>5.06</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>10</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.19</v>
+        <v>2.18</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>4</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-7</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="E39" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.58</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2966.9</v>
+        <v>3098.91</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-27.34</v>
+        <v>-149.11</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>0</v>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.43</v>
+        <v>6.49</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-34</v>
+        <v>-48</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=11.0bp [OK]
-HY OAS 5dd=8.0bp
+          <t>HY OAS 20dd=10.0bp [OK]
+HY OAS 5dd=4.0bp
 HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.1% [OK]
-SPY vs 200MA: above ($SPY=747.7100219726562, 200MA=689.7)
+FXY 5d=0.0% [OK]
+SPY vs 200MA: above ($SPY=745.4000244140625, 200MA=690.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-10 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>-3</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.31</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.56</v>
+        <v>4.54</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>10</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>4</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-7</v>
+        <v>-12</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-4</v>
+        <v>-9</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.58</v>
+        <v>3.53</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2013,7 +2013,7 @@
         <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>6</v>
+        <v>-2</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=10.0bp [OK]
-HY OAS 5dd=4.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=8.0bp [OK]
+HY OAS 5dd=5.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.0% [OK]
-SPY vs 200MA: above ($SPY=745.4000244140625, 200MA=690.2)
+FXY 5d=0.1% [OK]
+SPY vs 200MA: above ($SPY=751.7100219726562, 200MA=690.6)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-13 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.31</v>
+        <v>2.32</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-11</v>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.54</v>
+        <v>4.56</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>-1</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.05</v>
+        <v>5.06</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>4</v>
+        <v>-3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.53</v>
+        <v>3.55</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=8.0bp [OK]
+          <t>HY OAS 20dd=2.0bp [OK]
 HY OAS 5dd=5.0bp
-HYG 5d=0.2% [OK]
+HYG 5d=0.0% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.1% [OK]
-SPY vs 200MA: above ($SPY=751.7100219726562, 200MA=690.6)
+FXY 5d=-0.4% [OK]
+SPY vs 200MA: above ($SPY=754.9500122070312, 200MA=691.1)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-14 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>2</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.32</v>
+        <v>2.36</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-11</v>
+        <v>-20</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.56</v>
+        <v>4.62</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-1</v>
+        <v>-17</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.06</v>
+        <v>5.1</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-3</v>
+        <v>-15</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.55</v>
+        <v>3.6</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2013,7 +2013,7 @@
         <v>269</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=5.0bp
-HYG 5d=0.0% [OK]
+          <t>HY OAS 20dd=-3.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=-0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.4% [OK]
-SPY vs 200MA: above ($SPY=754.9500122070312, 200MA=691.1)
+FXY 5d=-0.2% [OK]
+SPY vs 200MA: above ($SPY=749.1699829101562, 200MA=691.6)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-15 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>6</v>
+        <v>-2</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.36</v>
+        <v>2.33</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-20</v>
+        <v>-16</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.62</v>
+        <v>4.58</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-17</v>
+        <v>-10</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.1</v>
+        <v>5.08</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-15</v>
+        <v>-11</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.22</v>
+        <v>2.21</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="E39" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
         <v>0</v>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.6</v>
+        <v>3.63</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-3.0bp [OK]
-HY OAS 5dd=3.0bp
-HYG 5d=-0.4% [OK]
+          <t>HY OAS 20dd=-1.0bp [OK]
+HY OAS 5dd=-5.0bp
+HYG 5d=-0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.2% [OK]
-SPY vs 200MA: above ($SPY=749.1699829101562, 200MA=691.6)
+FXY 5d=-0.1% [OK]
+SPY vs 200MA: above ($SPY=751.8300170898438, 200MA=692.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-16 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>0</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.33</v>
+        <v>2.32</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.58</v>
+        <v>4.55</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.63</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3098.91</v>
+        <v>3142.72</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-149.11</v>
+        <v>-176.96</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
         <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-1</v>
+        <v>-8</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-2</v>
+        <v>-10</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-48</v>
+        <v>-57</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=-5.0bp
-HYG 5d=-0.1% [OK]
+          <t>HY OAS 20dd=-8.0bp [OK]
+HY OAS 5dd=-1.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.1% [OK]
-SPY vs 200MA: above ($SPY=751.8300170898438, 200MA=692.0)
+FXY 5d=0.1% [OK]
+SPY vs 200MA: above ($SPY=754.8099975585938, 200MA=692.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-17 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F15" s="24" t="n">
         <v>-5</v>
@@ -978,7 +978,7 @@
         <v>29</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.32</v>
+        <v>2.35</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-17</v>
+        <v>-21</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.55</v>
+        <v>4.57</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-8</v>
+        <v>-14</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.08</v>
+        <v>5.09</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-11</v>
+        <v>-16</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.22</v>
+        <v>2.24</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F40" s="24" t="n">
         <v>1</v>
-      </c>
-      <c r="F40" s="24" t="n">
-        <v>5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2013,7 +2013,7 @@
         <v>271</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-10</v>
+        <v>-6</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,7 +2500,7 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F67" s="24" t="n">
         <v>-2</v>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-8.0bp [OK]
+          <t>HY OAS 20dd=-5.0bp [OK]
 HY OAS 5dd=-1.0bp
-HYG 5d=0.2% [OK]
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.1% [OK]
-SPY vs 200MA: above ($SPY=754.8099975585938, 200MA=692.5)
+FXY 5d=-0.1% [OK]
+SPY vs 200MA: above ($SPY=750.719970703125, 200MA=693.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-20 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-4</v>
+        <v>-12</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-3</v>
+        <v>-8</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-5</v>
+        <v>-15</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.35</v>
+        <v>2.31</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-21</v>
+        <v>-8</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.57</v>
+        <v>4.55</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-14</v>
+        <v>-6</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.09</v>
+        <v>5.06</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-16</v>
+        <v>-13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.59</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-5.0bp [OK]
-HY OAS 5dd=-1.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=-7.0bp [OK]
+HY OAS 5dd=-4.0bp
+HYG 5d=-0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.1% [OK]
-SPY vs 200MA: above ($SPY=750.719970703125, 200MA=693.0)
+FXY 5d=-0.4% [OK]
+SPY vs 200MA: above ($SPY=743.2899780273438, 200MA=693.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-21 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>78</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-15</v>
+        <v>-19</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>27</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.31</v>
+        <v>2.35</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-8</v>
+        <v>-14</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.55</v>
+        <v>4.6</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-6</v>
+        <v>-14</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.06</v>
+        <v>5.11</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-13</v>
+        <v>-21</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.25</v>
+        <v>2.26</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.22</v>
+        <v>2.24</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.59</v>
+        <v>3.57</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-7.0bp [OK]
-HY OAS 5dd=-4.0bp
-HYG 5d=-0.1% [OK]
+          <t>HY OAS 20dd=-4.0bp [OK]
+HY OAS 5dd=0.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.4% [OK]
-SPY vs 200MA: above ($SPY=743.2899780273438, 200MA=693.4)
+FXY 5d=0.0% [OK]
+SPY vs 200MA: above ($SPY=742.0900268554688, 200MA=693.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-22 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-19</v>
+        <v>-16</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-4</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-14</v>
+        <v>-9</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.6</v>
+        <v>4.63</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.11</v>
+        <v>5.13</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-21</v>
+        <v>-18</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.26</v>
+        <v>2.28</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>-7</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.57</v>
+        <v>3.61</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2013,7 +2013,7 @@
         <v>269</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-4.0bp [OK]
-HY OAS 5dd=0.0bp
-HYG 5d=0.2% [OK]
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=-0.0% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.0% [OK]
-SPY vs 200MA: above ($SPY=742.0900268554688, 200MA=693.8)
+FXY 5d=-0.6% [OK]
+SPY vs 200MA: above ($SPY=748.280029296875, 200MA=694.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-23 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-10</v>
+        <v>-2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Flattening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-16</v>
+        <v>-6</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.37</v>
+        <v>2.39</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.63</v>
+        <v>4.67</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-12</v>
+        <v>-17</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.13</v>
+        <v>5.15</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-18</v>
+        <v>-21</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.28</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.26</v>
+        <v>2.27</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>0</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.61</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>0</v>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3142.72</v>
+        <v>3062.15</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-176.96</v>
+        <v>-46.62</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
         <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.55</v>
+        <v>6.58</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-57</v>
+        <v>-58</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
+          <t>HY OAS 20dd=8.0bp [OK]
 HY OAS 5dd=3.0bp
-HYG 5d=-0.0% [OK]
+HYG 5d=-0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.6% [OK]
-SPY vs 200MA: above ($SPY=748.280029296875, 200MA=694.3)
+FXY 5d=-0.5% [OK]
+SPY vs 200MA: above ($SPY=747.4099731445312, 200MA=694.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-24 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.39</v>
+        <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.67</v>
+        <v>4.71</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-17</v>
+        <v>-30</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.15</v>
+        <v>5.17</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-21</v>
+        <v>-31</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.28</v>
+        <v>2.26</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=8.0bp [OK]
-HY OAS 5dd=3.0bp
-HYG 5d=-0.4% [OK]
+          <t>HY OAS 20dd=1.0bp [OK]
+HY OAS 5dd=-6.0bp
+HYG 5d=-0.7% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.5% [OK]
-SPY vs 200MA: above ($SPY=747.4099731445312, 200MA=694.7)
+FXY 5d=-0.8% [OK]
+SPY vs 200MA: above ($SPY=738.1799926757812, 200MA=695.1)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-27 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F11" s="24" t="n">
         <v>-2</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>-1</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-1</v>
@@ -1038,7 +1038,7 @@
         <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-20</v>
+        <v>-24</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.71</v>
+        <v>4.69</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.17</v>
+        <v>5.16</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.26</v>
+        <v>2.21</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.28</v>
+        <v>2.24</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-9</v>
+        <v>-5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>2</v>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=1.0bp [OK]
+          <t>HY OAS 20dd=4.0bp [OK]
 HY OAS 5dd=-6.0bp
-HYG 5d=-0.7% [OK]
+HYG 5d=-0.5% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=-0.8% [OK]
-SPY vs 200MA: above ($SPY=738.1799926757812, 200MA=695.1)
+SPY vs 200MA: above ($SPY=738.9299926757812, 200MA=695.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-28 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>47</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.43</v>
+        <v>2.44</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-24</v>
+        <v>-26</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.69</v>
+        <v>4.65</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-29</v>
+        <v>-27</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.16</v>
+        <v>5.12</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-30</v>
+        <v>-25</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.24</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=4.0bp [OK]
-HY OAS 5dd=-6.0bp
+          <t>HY OAS 20dd=-1.0bp [OK]
+HY OAS 5dd=-12.0bp
 HYG 5d=-0.5% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.8% [OK]
-SPY vs 200MA: above ($SPY=738.9299926757812, 200MA=695.4)
+FXY 5d=-0.9% [OK]
+SPY vs 200MA: above ($SPY=739.0900268554688, 200MA=695.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-29 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>3</v>
+        <v>-2</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-3</v>
+        <v>-7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-1</v>
+        <v>-7</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.44</v>
+        <v>2.41</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.65</v>
+        <v>4.61</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-27</v>
+        <v>-23</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.12</v>
+        <v>5.09</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-25</v>
+        <v>-23</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.2</v>
+        <v>2.26</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.24</v>
+        <v>2.28</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-1</v>
+        <v>-9</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=-12.0bp
-HYG 5d=-0.5% [OK]
+          <t>HY OAS 20dd=-9.0bp [OK]
+HY OAS 5dd=-15.0bp
+HYG 5d=-0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.9% [OK]
-SPY vs 200MA: above ($SPY=739.0900268554688, 200MA=695.8)
+FXY 5d=-0.4% [OK]
+SPY vs 200MA: above ($SPY=740.8599853515625, 200MA=696.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-30 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-2</v>
+        <v>-11</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-7</v>
+        <v>-15</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-7</v>
+        <v>-21</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.41</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-25</v>
+        <v>-21</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.61</v>
+        <v>4.67</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>-23</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.09</v>
+        <v>5.2</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-23</v>
+        <v>-29</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.26</v>
+        <v>2.27</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.28</v>
+        <v>2.3</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3062.15</v>
+        <v>2984.57</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-46.62</v>
+        <v>53.09</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-9</v>
+        <v>-13</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.58</v>
+        <v>6.66</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-58</v>
+        <v>-55</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-9.0bp [OK]
-HY OAS 5dd=-15.0bp
-HYG 5d=-0.3% [OK]
+          <t>HY OAS 20dd=-13.0bp [OK]
+HY OAS 5dd=-19.0bp
+HYG 5d=-0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.4% [OK]
-SPY vs 200MA: above ($SPY=740.8599853515625, 200MA=696.2)
+FXY 5d=-0.2% [OK]
+SPY vs 200MA: above ($SPY=729.4600219726562, 200MA=696.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-07-31 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>83</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>45</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>98</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-21</v>
+        <v>-18</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.41</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-21</v>
+        <v>-16</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.67</v>
+        <v>4.68</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-23</v>
+        <v>-20</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.2</v>
+        <v>5.21</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-29</v>
+        <v>-24</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.3</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-5</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-13</v>
+        <v>-9</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>0</v>
+        <v>-14</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-13.0bp [OK]
-HY OAS 5dd=-19.0bp
-HYG 5d=-0.4% [OK]
+          <t>HY OAS 20dd=-9.0bp [OK]
+HY OAS 5dd=-7.0bp
+HYG 5d=0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.2% [OK]
-SPY vs 200MA: above ($SPY=729.4600219726562, 200MA=696.5)
+FXY 5d=2.8% [TRIGGERED]
+SPY vs 200MA: above ($SPY=741.6900024414062, 200MA=697.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-03 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-18</v>
+        <v>-15</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.41</v>
+        <v>2.47</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-16</v>
+        <v>-21</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.68</v>
+        <v>4.75</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-20</v>
+        <v>-26</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.21</v>
+        <v>5.27</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-24</v>
+        <v>-29</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2918,8 +2918,8 @@
 HY OAS 5dd=-7.0bp
 HYG 5d=0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=2.8% [TRIGGERED]
-SPY vs 200MA: above ($SPY=741.6900024414062, 200MA=697.0)
+FXY 5d=2.9% [TRIGGERED]
+SPY vs 200MA: above ($SPY=747.030029296875, 200MA=697.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-04 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.47</v>
+        <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-21</v>
+        <v>-19</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.75</v>
+        <v>4.7</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-26</v>
+        <v>-22</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.27</v>
+        <v>5.23</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-29</v>
+        <v>-24</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.27</v>
+        <v>2.23</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>2.27</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>-2</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>-2</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-2</v>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-9.0bp [OK]
-HY OAS 5dd=-7.0bp
-HYG 5d=0.3% [OK]
+          <t>HY OAS 20dd=-6.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=0.5% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=2.9% [TRIGGERED]
-SPY vs 200MA: above ($SPY=747.030029296875, 200MA=697.4)
+FXY 5d=4.4% [TRIGGERED]
+SPY vs 200MA: above ($SPY=757.6699829101562, 200MA=697.9)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-05 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -978,7 +978,7 @@
         <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.43</v>
+        <v>2.4</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-19</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.7</v>
+        <v>4.63</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-22</v>
+        <v>-8</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.23</v>
+        <v>5.18</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-24</v>
+        <v>-13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.27</v>
+        <v>2.26</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="F51" s="24" t="n">
         <v>-6</v>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2915,11 +2915,11 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=-6.0bp [OK]
-HY OAS 5dd=3.0bp
-HYG 5d=0.5% [OK]
+HY OAS 5dd=11.0bp
+HYG 5d=0.6% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=4.4% [TRIGGERED]
-SPY vs 200MA: above ($SPY=757.6699829101562, 200MA=697.9)
+FXY 5d=3.8% [TRIGGERED]
+SPY vs 200MA: above ($SPY=771.3300170898438, 200MA=698.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-10 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-8</v>
+        <v>-15</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.43</v>
+        <v>2.4</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.69</v>
+        <v>4.65</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-15</v>
+        <v>-9</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.22</v>
+        <v>5.19</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-17</v>
+        <v>-13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.25</v>
+        <v>2.29</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.28</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-12</v>
+        <v>-7</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-11</v>
+        <v>-6</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-12</v>
+        <v>-7</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
         <v>-1</v>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2915,11 +2915,11 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=13.0bp
-HYG 5d=0.5% [OK]
+HY OAS 5dd=15.0bp
+HYG 5d=0.6% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.5% [OK]
-SPY vs 200MA: above ($SPY=768.5599975585938, 200MA=699.6)
+FXY 5d=1.0% [OK]
+SPY vs 200MA: above ($SPY=773.260009765625, 200MA=700.1)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-11 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>84</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-8</v>
+        <v>-11</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F13" s="24" t="n">
         <v>-11</v>
@@ -949,7 +949,7 @@
         <v>100</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-15</v>
+        <v>-16</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.4</v>
+        <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.65</v>
+        <v>4.72</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.19</v>
+        <v>5.25</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-13</v>
+        <v>-15</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.31</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>-3</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>-7</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2915,11 +2915,11 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=15.0bp
-HYG 5d=0.6% [OK]
+HY OAS 5dd=8.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=1.0% [OK]
-SPY vs 200MA: above ($SPY=773.260009765625, 200MA=700.1)
+FXY 5d=-1.5% [OK]
+SPY vs 200MA: above ($SPY=773.030029296875, 200MA=700.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-12 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Flattening</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-16</v>
+        <v>-12</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>31</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.72</v>
+        <v>4.7</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-10</v>
+        <v>-12</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.25</v>
+        <v>5.24</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-15</v>
+        <v>-16</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.27</v>
+        <v>2.26</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>2.28</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.63</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>0</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=8.0bp
-HYG 5d=0.2% [OK]
+          <t>HY OAS 20dd=0.0bp [OK]
+HY OAS 5dd=1.0bp
+HYG 5d=-0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-1.5% [OK]
-SPY vs 200MA: above ($SPY=773.030029296875, 200MA=700.7)
+FXY 5d=-0.9% [OK]
+SPY vs 200MA: above ($SPY=770.5599975585938, 200MA=701.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-13 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1845" yWindow="2460" windowWidth="17910" windowHeight="9870" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily Input" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="字段说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="示例 2026-05-17" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026-05-18" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Input" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例 2026-05-17" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-05-18" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>48</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.43</v>
+        <v>2.42</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-10</v>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.7</v>
+        <v>4.68</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.26</v>
+        <v>2.24</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>-7</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2993.35</v>
+        <v>2944.06</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>26.65</v>
+        <v>49.9</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F51" s="24" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>138</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.69</v>
+        <v>6.67</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-47</v>
+        <v>-29</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2915,11 +2915,11 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=0.0bp [OK]
-HY OAS 5dd=1.0bp
-HYG 5d=-0.1% [OK]
+HY OAS 5dd=4.0bp
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.9% [OK]
-SPY vs 200MA: above ($SPY=770.5599975585938, 200MA=701.2)
+FXY 5d=-1.1% [OK]
+SPY vs 200MA: above ($SPY=772.489990234375, 200MA=701.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-14 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>48</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-9</v>
+        <v>-13</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.42</v>
+        <v>2.39</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.68</v>
+        <v>4.63</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-13</v>
+        <v>-6</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.24</v>
+        <v>5.21</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-16</v>
+        <v>-12</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.24</v>
+        <v>2.27</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.27</v>
+        <v>2.3</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-7</v>
+        <v>-9</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-3</v>
+        <v>-8</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2915,11 +2915,11 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=0.0bp [OK]
-HY OAS 5dd=4.0bp
-HYG 5d=0.1% [OK]
+HY OAS 5dd=0.0bp
+HYG 5d=0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-1.1% [OK]
-SPY vs 200MA: above ($SPY=772.489990234375, 200MA=701.7)
+FXY 5d=-0.6% [OK]
+SPY vs 200MA: above ($SPY=777.8800048828125, 200MA=702.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-17 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>89</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-8</v>
+        <v>-11</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>-6</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-7</v>
+        <v>-14</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-13</v>
+        <v>-20</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.39</v>
+        <v>2.41</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-4</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.63</v>
+        <v>4.68</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-6</v>
+        <v>-13</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.21</v>
+        <v>5.25</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-12</v>
+        <v>-19</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>-3</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>-9</v>
@@ -1624,7 +1624,7 @@
         <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-1</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=0.0bp [OK]
-HY OAS 5dd=0.0bp
-HYG 5d=0.4% [OK]
+          <t>HY OAS 20dd=6.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.6% [OK]
-SPY vs 200MA: above ($SPY=777.8800048828125, 200MA=702.3)
+FXY 5d=-1.1% [OK]
+SPY vs 200MA: above ($SPY=776.3400268554688, 200MA=702.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-18 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-11</v>
+        <v>-15</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F13" s="24" t="n">
         <v>-14</v>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-20</v>
+        <v>-22</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.41</v>
+        <v>2.44</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.68</v>
+        <v>4.72</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.25</v>
+        <v>5.31</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-19</v>
+        <v>-20</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.28</v>
+        <v>2.3</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>-9</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=6.0bp [OK]
-HY OAS 5dd=3.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=-1.0bp [OK]
+HY OAS 5dd=0.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-1.1% [OK]
-SPY vs 200MA: above ($SPY=776.3400268554688, 200MA=702.8)
+FXY 5d=-0.2% [OK]
+SPY vs 200MA: above ($SPY=772.6699829101562, 200MA=703.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-19 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F11" s="24" t="n">
         <v>-15</v>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Flattening</t>
+          <t>Bear Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F15" s="24" t="n">
         <v>-22</v>
@@ -978,7 +978,7 @@
         <v>34</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.44</v>
+        <v>2.41</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-9</v>
+        <v>-4</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.72</v>
+        <v>4.71</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.31</v>
+        <v>5.28</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-20</v>
+        <v>-15</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.3</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.32</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-9</v>
+        <v>-4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-9</v>
+        <v>-4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-9</v>
+        <v>-4</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-1</v>
+        <v>-6</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=0.0bp
-HYG 5d=0.2% [OK]
+          <t>HY OAS 20dd=-6.0bp [OK]
+HY OAS 5dd=-3.0bp
+HYG 5d=0.0% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.2% [OK]
-SPY vs 200MA: above ($SPY=772.6699829101562, 200MA=703.2)
+FXY 5d=-0.3% [OK]
+SPY vs 200MA: above ($SPY=767.4500122070312, 200MA=703.6)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-20 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-15</v>
+        <v>-10</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-15</v>
+        <v>-10</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-22</v>
+        <v>-16</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.41</v>
+        <v>2.35</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.71</v>
+        <v>4.65</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-8</v>
+        <v>2</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.28</v>
+        <v>5.19</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-15</v>
+        <v>-4</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-2</v>
+        <v>-6</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>0</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>-4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2944.06</v>
+        <v>2935.29</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>49.9</v>
+        <v>91.42</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.67</v>
+        <v>6.65</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-29</v>
+        <v>-19</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-6.0bp [OK]
-HY OAS 5dd=-3.0bp
-HYG 5d=0.0% [OK]
+          <t>HY OAS 20dd=-5.0bp [OK]
+HY OAS 5dd=-2.0bp
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.3% [OK]
-SPY vs 200MA: above ($SPY=767.4500122070312, 200MA=703.6)
+FXY 5d=0.9% [OK]
+SPY vs 200MA: above ($SPY=769.0599975585938, 200MA=704.1)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-21 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>84</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-10</v>
+        <v>-13</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>54</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-10</v>
+        <v>-16</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-16</v>
+        <v>-24</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>30</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.35</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.65</v>
+        <v>4.69</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>2</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.19</v>
+        <v>5.23</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-5</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>141</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-8</v>
+        <v>19</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-5.0bp [OK]
-HY OAS 5dd=-2.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=-4.0bp
+HYG 5d=-0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.9% [OK]
-SPY vs 200MA: above ($SPY=769.0599975585938, 200MA=704.1)
+FXY 5d=0.2% [OK]
+SPY vs 200MA: above ($SPY=762.5999755859375, 200MA=704.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-24 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>MON</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>84</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-13</v>
+        <v>-11</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>50</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-16</v>
+        <v>-14</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-24</v>
+        <v>-20</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-5</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.35</v>
+        <v>2.4</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.69</v>
+        <v>4.74</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>2</v>
+        <v>-5</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.23</v>
+        <v>5.27</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-8</v>
+        <v>-11</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.63</v>
+        <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=-4.0bp
-HYG 5d=-0.3% [OK]
+          <t>HY OAS 20dd=9.0bp [OK]
+HY OAS 5dd=-3.0bp
+HYG 5d=-0.1% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=0.2% [OK]
-SPY vs 200MA: above ($SPY=762.5999755859375, 200MA=704.5)
+SPY vs 200MA: above ($SPY=765.719970703125, 200MA=705.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-25 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>MON</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.4</v>
+        <v>2.38</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>-5</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.27</v>
+        <v>5.23</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>-11</v>
@@ -1353,7 +1353,7 @@
         <v>2.32</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
         <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=9.0bp [OK]
-HY OAS 5dd=-3.0bp
-HYG 5d=-0.1% [OK]
+          <t>HY OAS 20dd=12.0bp [OK]
+HY OAS 5dd=1.0bp
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=0.2% [OK]
-SPY vs 200MA: above ($SPY=765.719970703125, 200MA=705.0)
+SPY vs 200MA: above ($SPY=763.469970703125, 200MA=705.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-27 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>82</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>53</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F13" s="24" t="n">
         <v>-12</v>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>29</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.38</v>
+        <v>2.32</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.7</v>
+        <v>4.64</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.23</v>
+        <v>5.17</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.32</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-12</v>
+        <v>-6</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-9</v>
+        <v>-5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>-1</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>-1</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-1</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>7</v>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=12.0bp [OK]
-HY OAS 5dd=1.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=14.0bp [OK]
+HY OAS 5dd=5.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.2% [OK]
-SPY vs 200MA: above ($SPY=763.469970703125, 200MA=705.5)
+FXY 5d=-0.8% [OK]
+SPY vs 200MA: above ($SPY=766.0800170898438, 200MA=706.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-28 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-8</v>
+        <v>2</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-5</v>
+        <v>1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>47</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-12</v>
+        <v>-2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bear Flattening</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-17</v>
+        <v>-1</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>29</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.64</v>
+        <v>4.66</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.17</v>
+        <v>5.18</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-8</v>
+        <v>2</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>-6</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>-5</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>1</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.66</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2935.29</v>
+        <v>2924.94</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>91.42</v>
+        <v>191.31</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.65</v>
+        <v>6.66</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-19</v>
+        <v>-29</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=14.0bp [OK]
-HY OAS 5dd=5.0bp
-HYG 5d=0.2% [OK]
+          <t>HY OAS 20dd=20.0bp [OK]
+HY OAS 5dd=6.0bp
+HYG 5d=0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.8% [OK]
-SPY vs 200MA: above ($SPY=766.0800170898438, 200MA=706.4)
+FXY 5d=-0.3% [OK]
+SPY vs 200MA: above ($SPY=771.0999755859375, 200MA=707.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-08-29 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Bear Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.66</v>
+        <v>4.67</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>1</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.18</v>
+        <v>5.19</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>2</v>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.33</v>
+        <v>2.31</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.35</v>
+        <v>2.32</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>1</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=20.0bp [OK]
-HY OAS 5dd=6.0bp
-HYG 5d=0.4% [OK]
+          <t>HY OAS 20dd=21.0bp [TRIGGERED]
+HY OAS 5dd=12.0bp
+HYG 5d=0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.3% [OK]
-SPY vs 200MA: above ($SPY=771.0999755859375, 200MA=707.0)
+FXY 5d=-0.8% [OK]
+SPY vs 200MA: above ($SPY=769.3499755859375, 200MA=707.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-02 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.44</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.75</v>
+        <v>4.79</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-5</v>
+        <v>-16</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.25</v>
+        <v>5.27</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-2</v>
+        <v>-9</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>-12</v>
@@ -1436,7 +1436,7 @@
         <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.68</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=15.0bp [OK]
-HY OAS 5dd=6.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=8.0bp [OK]
+HY OAS 5dd=5.0bp
+HYG 5d=-0.5% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.4% [OK]
-SPY vs 200MA: above ($SPY=767.0499877929688, 200MA=707.9)
+FXY 5d=-0.7% [OK]
+SPY vs 200MA: above ($SPY=761.780029296875, 200MA=708.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-03 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>40</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -949,7 +949,7 @@
         <v>88</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.44</v>
+        <v>2.45</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-4</v>
@@ -1096,7 +1096,7 @@
         <v>5.27</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2924.94</v>
+        <v>2894.53</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>191.31</v>
+        <v>235.06</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.66</v>
+        <v>6.71</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-29</v>
+        <v>-41</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=8.0bp [OK]
-HY OAS 5dd=5.0bp
-HYG 5d=-0.5% [OK]
+          <t>HY OAS 20dd=9.0bp [OK]
+HY OAS 5dd=1.0bp
+HYG 5d=-0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.7% [OK]
-SPY vs 200MA: above ($SPY=761.780029296875, 200MA=708.3)
+FXY 5d=0.3% [OK]
+SPY vs 200MA: above ($SPY=765.1599731445312, 200MA=708.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-04 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>73</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>48</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.45</v>
+        <v>2.42</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.79</v>
+        <v>4.77</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-16</v>
+        <v>-8</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.27</v>
+        <v>5.25</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-10</v>
+        <v>-3</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>-1</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>-1</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.66</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-1</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>138</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=9.0bp [OK]
-HY OAS 5dd=1.0bp
-HYG 5d=-0.4% [OK]
+          <t>HY OAS 20dd=6.0bp [OK]
+HY OAS 5dd=-2.0bp
+HYG 5d=-0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.3% [OK]
-SPY vs 200MA: above ($SPY=765.1599731445312, 200MA=708.8)
+FXY 5d=2.4% [OK]
+SPY vs 200MA: above ($SPY=773.1699829101562, 200MA=709.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>